<commit_message>
replaced spice powder and fixed icons
</commit_message>
<xml_diff>
--- a/data/config/export/main/asset/assets_includes/items/items.xlsx
+++ b/data/config/export/main/asset/assets_includes/items/items.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Max\Documents\Anno 1800\mods\[Addon] Return to the Orient\data\config\export\main\asset\assets_includes\items\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55536D3D-39B7-4930-835E-069FB3DB25DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19EB6558-6075-454C-9179-ED5DA71BFC6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="5235" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -864,7 +864,7 @@
         <v>36</v>
       </c>
       <c r="C2" t="str">
-        <f>"&lt;Item&gt;
+        <f t="shared" ref="C2:C43" si="0">"&lt;Item&gt;
             &lt;ItemLink&gt;" &amp; B2 &amp; "&lt;/ItemLink&gt;
         &lt;/Item&gt;"</f>
         <v>&lt;Item&gt;
@@ -895,9 +895,7 @@
         <v>58</v>
       </c>
       <c r="C3" t="str">
-        <f>"&lt;Item&gt;
-            &lt;ItemLink&gt;" &amp; B3 &amp; "&lt;/ItemLink&gt;
-        &lt;/Item&gt;"</f>
+        <f t="shared" si="0"/>
         <v>&lt;Item&gt;
             &lt;ItemLink&gt;1404000894&lt;/ItemLink&gt;
         &lt;/Item&gt;</v>
@@ -926,9 +924,7 @@
         <v>115</v>
       </c>
       <c r="C4" t="str">
-        <f>"&lt;Item&gt;
-            &lt;ItemLink&gt;" &amp; B4 &amp; "&lt;/ItemLink&gt;
-        &lt;/Item&gt;"</f>
+        <f t="shared" si="0"/>
         <v>&lt;Item&gt;
             &lt;ItemLink&gt;1404000905&lt;/ItemLink&gt;
         &lt;/Item&gt;</v>
@@ -957,9 +953,7 @@
         <v>7</v>
       </c>
       <c r="C5" t="str">
-        <f>"&lt;Item&gt;
-            &lt;ItemLink&gt;" &amp; B5 &amp; "&lt;/ItemLink&gt;
-        &lt;/Item&gt;"</f>
+        <f t="shared" si="0"/>
         <v>&lt;Item&gt;
             &lt;ItemLink&gt;1404000921&lt;/ItemLink&gt;
         &lt;/Item&gt;</v>
@@ -988,9 +982,7 @@
         <v>27</v>
       </c>
       <c r="C6" t="str">
-        <f>"&lt;Item&gt;
-            &lt;ItemLink&gt;" &amp; B6 &amp; "&lt;/ItemLink&gt;
-        &lt;/Item&gt;"</f>
+        <f t="shared" si="0"/>
         <v>&lt;Item&gt;
             &lt;ItemLink&gt;1404000927&lt;/ItemLink&gt;
         &lt;/Item&gt;</v>
@@ -1019,9 +1011,7 @@
         <v>121</v>
       </c>
       <c r="C7" t="str">
-        <f>"&lt;Item&gt;
-            &lt;ItemLink&gt;" &amp; B7 &amp; "&lt;/ItemLink&gt;
-        &lt;/Item&gt;"</f>
+        <f t="shared" si="0"/>
         <v>&lt;Item&gt;
             &lt;ItemLink&gt;1404000920&lt;/ItemLink&gt;
         &lt;/Item&gt;</v>
@@ -1050,9 +1040,7 @@
         <v>33</v>
       </c>
       <c r="C8" t="str">
-        <f>"&lt;Item&gt;
-            &lt;ItemLink&gt;" &amp; B8 &amp; "&lt;/ItemLink&gt;
-        &lt;/Item&gt;"</f>
+        <f t="shared" si="0"/>
         <v>&lt;Item&gt;
             &lt;ItemLink&gt;1404000925&lt;/ItemLink&gt;
         &lt;/Item&gt;</v>
@@ -1081,9 +1069,7 @@
         <v>46</v>
       </c>
       <c r="C9" t="str">
-        <f>"&lt;Item&gt;
-            &lt;ItemLink&gt;" &amp; B9 &amp; "&lt;/ItemLink&gt;
-        &lt;/Item&gt;"</f>
+        <f t="shared" si="0"/>
         <v>&lt;Item&gt;
             &lt;ItemLink&gt;1404000890&lt;/ItemLink&gt;
         &lt;/Item&gt;</v>
@@ -1112,9 +1098,7 @@
         <v>106</v>
       </c>
       <c r="C10" t="str">
-        <f>"&lt;Item&gt;
-            &lt;ItemLink&gt;" &amp; B10 &amp; "&lt;/ItemLink&gt;
-        &lt;/Item&gt;"</f>
+        <f t="shared" si="0"/>
         <v>&lt;Item&gt;
             &lt;ItemLink&gt;1404000919&lt;/ItemLink&gt;
         &lt;/Item&gt;</v>
@@ -1143,9 +1127,7 @@
         <v>112</v>
       </c>
       <c r="C11" t="str">
-        <f>"&lt;Item&gt;
-            &lt;ItemLink&gt;" &amp; B11 &amp; "&lt;/ItemLink&gt;
-        &lt;/Item&gt;"</f>
+        <f t="shared" si="0"/>
         <v>&lt;Item&gt;
             &lt;ItemLink&gt;1404000897&lt;/ItemLink&gt;
         &lt;/Item&gt;</v>
@@ -1174,9 +1156,7 @@
         <v>124</v>
       </c>
       <c r="C12" t="str">
-        <f>"&lt;Item&gt;
-            &lt;ItemLink&gt;" &amp; B12 &amp; "&lt;/ItemLink&gt;
-        &lt;/Item&gt;"</f>
+        <f t="shared" si="0"/>
         <v>&lt;Item&gt;
             &lt;ItemLink&gt;1404000908&lt;/ItemLink&gt;
         &lt;/Item&gt;</v>
@@ -1205,9 +1185,7 @@
         <v>109</v>
       </c>
       <c r="C13" t="str">
-        <f>"&lt;Item&gt;
-            &lt;ItemLink&gt;" &amp; B13 &amp; "&lt;/ItemLink&gt;
-        &lt;/Item&gt;"</f>
+        <f t="shared" si="0"/>
         <v>&lt;Item&gt;
             &lt;ItemLink&gt;1404000910&lt;/ItemLink&gt;
         &lt;/Item&gt;</v>
@@ -1236,9 +1214,7 @@
         <v>73</v>
       </c>
       <c r="C14" t="str">
-        <f>"&lt;Item&gt;
-            &lt;ItemLink&gt;" &amp; B14 &amp; "&lt;/ItemLink&gt;
-        &lt;/Item&gt;"</f>
+        <f t="shared" si="0"/>
         <v>&lt;Item&gt;
             &lt;ItemLink&gt;1404000914&lt;/ItemLink&gt;
         &lt;/Item&gt;</v>
@@ -1261,27 +1237,27 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="B15" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="C15" t="str">
         <f>"&lt;Item&gt;
             &lt;ItemLink&gt;" &amp; B15 &amp; "&lt;/ItemLink&gt;
         &lt;/Item&gt;"</f>
         <v>&lt;Item&gt;
-            &lt;ItemLink&gt;1404000889&lt;/ItemLink&gt;
+            &lt;ItemLink&gt;1404000888&lt;/ItemLink&gt;
         &lt;/Item&gt;</v>
       </c>
       <c r="D15" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="E15" t="s">
         <v>9</v>
       </c>
       <c r="F15" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="G15" t="s">
         <v>9</v>
@@ -1292,21 +1268,21 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>78</v>
+        <v>48</v>
       </c>
       <c r="B16" t="s">
-        <v>79</v>
+        <v>49</v>
       </c>
       <c r="C16" t="str">
         <f>"&lt;Item&gt;
             &lt;ItemLink&gt;" &amp; B16 &amp; "&lt;/ItemLink&gt;
         &lt;/Item&gt;"</f>
         <v>&lt;Item&gt;
-            &lt;ItemLink&gt;1404000902&lt;/ItemLink&gt;
+            &lt;ItemLink&gt;1404000889&lt;/ItemLink&gt;
         &lt;/Item&gt;</v>
       </c>
       <c r="D16" t="s">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="E16" t="s">
         <v>9</v>
@@ -1323,27 +1299,27 @@
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>69</v>
+        <v>42</v>
       </c>
       <c r="B17" t="s">
-        <v>70</v>
+        <v>43</v>
       </c>
       <c r="C17" t="str">
         <f>"&lt;Item&gt;
             &lt;ItemLink&gt;" &amp; B17 &amp; "&lt;/ItemLink&gt;
         &lt;/Item&gt;"</f>
         <v>&lt;Item&gt;
-            &lt;ItemLink&gt;1404000906&lt;/ItemLink&gt;
+            &lt;ItemLink&gt;1404000891&lt;/ItemLink&gt;
         &lt;/Item&gt;</v>
       </c>
       <c r="D17" t="s">
-        <v>71</v>
+        <v>44</v>
       </c>
       <c r="E17" t="s">
         <v>9</v>
       </c>
       <c r="F17" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="G17" t="s">
         <v>9</v>
@@ -1354,27 +1330,27 @@
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>129</v>
+        <v>54</v>
       </c>
       <c r="B18" t="s">
-        <v>130</v>
+        <v>55</v>
       </c>
       <c r="C18" t="str">
         <f>"&lt;Item&gt;
             &lt;ItemLink&gt;" &amp; B18 &amp; "&lt;/ItemLink&gt;
         &lt;/Item&gt;"</f>
         <v>&lt;Item&gt;
-            &lt;ItemLink&gt;1404000895&lt;/ItemLink&gt;
+            &lt;ItemLink&gt;1404000893&lt;/ItemLink&gt;
         &lt;/Item&gt;</v>
       </c>
       <c r="D18" t="s">
-        <v>131</v>
+        <v>56</v>
       </c>
       <c r="E18" t="s">
         <v>9</v>
       </c>
       <c r="F18" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="G18" t="s">
         <v>9</v>
@@ -1385,21 +1361,21 @@
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>81</v>
+        <v>129</v>
       </c>
       <c r="B19" t="s">
-        <v>82</v>
+        <v>130</v>
       </c>
       <c r="C19" t="str">
         <f>"&lt;Item&gt;
             &lt;ItemLink&gt;" &amp; B19 &amp; "&lt;/ItemLink&gt;
         &lt;/Item&gt;"</f>
         <v>&lt;Item&gt;
-            &lt;ItemLink&gt;1404000903&lt;/ItemLink&gt;
+            &lt;ItemLink&gt;1404000895&lt;/ItemLink&gt;
         &lt;/Item&gt;</v>
       </c>
       <c r="D19" t="s">
-        <v>83</v>
+        <v>131</v>
       </c>
       <c r="E19" t="s">
         <v>9</v>
@@ -1416,27 +1392,27 @@
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>87</v>
+        <v>60</v>
       </c>
       <c r="B20" t="s">
-        <v>88</v>
+        <v>61</v>
       </c>
       <c r="C20" t="str">
         <f>"&lt;Item&gt;
             &lt;ItemLink&gt;" &amp; B20 &amp; "&lt;/ItemLink&gt;
         &lt;/Item&gt;"</f>
         <v>&lt;Item&gt;
-            &lt;ItemLink&gt;1404000911&lt;/ItemLink&gt;
+            &lt;ItemLink&gt;1404000896&lt;/ItemLink&gt;
         &lt;/Item&gt;</v>
       </c>
       <c r="D20" t="s">
-        <v>89</v>
+        <v>62</v>
       </c>
       <c r="E20" t="s">
         <v>9</v>
       </c>
       <c r="F20" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="G20" t="s">
         <v>9</v>
@@ -1447,27 +1423,27 @@
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>126</v>
+        <v>75</v>
       </c>
       <c r="B21" t="s">
-        <v>127</v>
+        <v>76</v>
       </c>
       <c r="C21" t="str">
         <f>"&lt;Item&gt;
             &lt;ItemLink&gt;" &amp; B21 &amp; "&lt;/ItemLink&gt;
         &lt;/Item&gt;"</f>
         <v>&lt;Item&gt;
-            &lt;ItemLink&gt;1404000912&lt;/ItemLink&gt;
+            &lt;ItemLink&gt;1404000898&lt;/ItemLink&gt;
         &lt;/Item&gt;</v>
       </c>
       <c r="D21" t="s">
-        <v>128</v>
+        <v>77</v>
       </c>
       <c r="E21" t="s">
         <v>9</v>
       </c>
       <c r="F21" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="G21" t="s">
         <v>9</v>
@@ -1478,27 +1454,27 @@
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>117</v>
+        <v>93</v>
       </c>
       <c r="B22" t="s">
-        <v>118</v>
+        <v>94</v>
       </c>
       <c r="C22" t="str">
         <f>"&lt;Item&gt;
             &lt;ItemLink&gt;" &amp; B22 &amp; "&lt;/ItemLink&gt;
         &lt;/Item&gt;"</f>
         <v>&lt;Item&gt;
-            &lt;ItemLink&gt;1404000916&lt;/ItemLink&gt;
+            &lt;ItemLink&gt;1404000899&lt;/ItemLink&gt;
         &lt;/Item&gt;</v>
       </c>
       <c r="D22" t="s">
-        <v>119</v>
+        <v>95</v>
       </c>
       <c r="E22" t="s">
         <v>9</v>
       </c>
       <c r="F22" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="G22" t="s">
         <v>9</v>
@@ -1509,21 +1485,21 @@
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>39</v>
+        <v>90</v>
       </c>
       <c r="B23" t="s">
-        <v>40</v>
+        <v>91</v>
       </c>
       <c r="C23" t="str">
         <f>"&lt;Item&gt;
             &lt;ItemLink&gt;" &amp; B23 &amp; "&lt;/ItemLink&gt;
         &lt;/Item&gt;"</f>
         <v>&lt;Item&gt;
-            &lt;ItemLink&gt;1404000888&lt;/ItemLink&gt;
+            &lt;ItemLink&gt;1404000900&lt;/ItemLink&gt;
         &lt;/Item&gt;</v>
       </c>
       <c r="D23" t="s">
-        <v>41</v>
+        <v>92</v>
       </c>
       <c r="E23" t="s">
         <v>9</v>
@@ -1540,27 +1516,27 @@
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="B24" t="s">
-        <v>43</v>
+        <v>64</v>
       </c>
       <c r="C24" t="str">
         <f>"&lt;Item&gt;
             &lt;ItemLink&gt;" &amp; B24 &amp; "&lt;/ItemLink&gt;
         &lt;/Item&gt;"</f>
         <v>&lt;Item&gt;
-            &lt;ItemLink&gt;1404000891&lt;/ItemLink&gt;
+            &lt;ItemLink&gt;1404000901&lt;/ItemLink&gt;
         &lt;/Item&gt;</v>
       </c>
       <c r="D24" t="s">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="E24" t="s">
         <v>9</v>
       </c>
       <c r="F24" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="G24" t="s">
         <v>9</v>
@@ -1571,27 +1547,27 @@
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>60</v>
+        <v>78</v>
       </c>
       <c r="B25" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="C25" t="str">
         <f>"&lt;Item&gt;
             &lt;ItemLink&gt;" &amp; B25 &amp; "&lt;/ItemLink&gt;
         &lt;/Item&gt;"</f>
         <v>&lt;Item&gt;
-            &lt;ItemLink&gt;1404000896&lt;/ItemLink&gt;
+            &lt;ItemLink&gt;1404000902&lt;/ItemLink&gt;
         &lt;/Item&gt;</v>
       </c>
       <c r="D25" t="s">
-        <v>62</v>
+        <v>80</v>
       </c>
       <c r="E25" t="s">
         <v>9</v>
       </c>
       <c r="F25" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="G25" t="s">
         <v>9</v>
@@ -1602,27 +1578,27 @@
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="B26" t="s">
-        <v>94</v>
+        <v>82</v>
       </c>
       <c r="C26" t="str">
         <f>"&lt;Item&gt;
             &lt;ItemLink&gt;" &amp; B26 &amp; "&lt;/ItemLink&gt;
         &lt;/Item&gt;"</f>
         <v>&lt;Item&gt;
-            &lt;ItemLink&gt;1404000899&lt;/ItemLink&gt;
+            &lt;ItemLink&gt;1404000903&lt;/ItemLink&gt;
         &lt;/Item&gt;</v>
       </c>
       <c r="D26" t="s">
-        <v>95</v>
+        <v>83</v>
       </c>
       <c r="E26" t="s">
         <v>9</v>
       </c>
       <c r="F26" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="G26" t="s">
         <v>9</v>
@@ -1633,27 +1609,27 @@
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>90</v>
+        <v>69</v>
       </c>
       <c r="B27" t="s">
-        <v>91</v>
+        <v>70</v>
       </c>
       <c r="C27" t="str">
         <f>"&lt;Item&gt;
             &lt;ItemLink&gt;" &amp; B27 &amp; "&lt;/ItemLink&gt;
         &lt;/Item&gt;"</f>
         <v>&lt;Item&gt;
-            &lt;ItemLink&gt;1404000900&lt;/ItemLink&gt;
+            &lt;ItemLink&gt;1404000906&lt;/ItemLink&gt;
         &lt;/Item&gt;</v>
       </c>
       <c r="D27" t="s">
-        <v>92</v>
+        <v>71</v>
       </c>
       <c r="E27" t="s">
         <v>9</v>
       </c>
       <c r="F27" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="G27" t="s">
         <v>9</v>
@@ -1726,27 +1702,27 @@
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>102</v>
+        <v>87</v>
       </c>
       <c r="B30" t="s">
-        <v>103</v>
+        <v>88</v>
       </c>
       <c r="C30" t="str">
         <f>"&lt;Item&gt;
             &lt;ItemLink&gt;" &amp; B30 &amp; "&lt;/ItemLink&gt;
         &lt;/Item&gt;"</f>
         <v>&lt;Item&gt;
-            &lt;ItemLink&gt;1404000915&lt;/ItemLink&gt;
+            &lt;ItemLink&gt;1404000911&lt;/ItemLink&gt;
         &lt;/Item&gt;</v>
       </c>
       <c r="D30" t="s">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="E30" t="s">
         <v>9</v>
       </c>
       <c r="F30" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="G30" t="s">
         <v>9</v>
@@ -1757,27 +1733,27 @@
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>66</v>
+        <v>126</v>
       </c>
       <c r="B31" t="s">
-        <v>67</v>
+        <v>127</v>
       </c>
       <c r="C31" t="str">
         <f>"&lt;Item&gt;
             &lt;ItemLink&gt;" &amp; B31 &amp; "&lt;/ItemLink&gt;
         &lt;/Item&gt;"</f>
         <v>&lt;Item&gt;
-            &lt;ItemLink&gt;1404000917&lt;/ItemLink&gt;
+            &lt;ItemLink&gt;1404000912&lt;/ItemLink&gt;
         &lt;/Item&gt;</v>
       </c>
       <c r="D31" t="s">
-        <v>68</v>
+        <v>128</v>
       </c>
       <c r="E31" t="s">
         <v>9</v>
       </c>
       <c r="F31" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="G31" t="s">
         <v>9</v>
@@ -1788,21 +1764,21 @@
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>54</v>
+        <v>96</v>
       </c>
       <c r="B32" t="s">
-        <v>55</v>
+        <v>97</v>
       </c>
       <c r="C32" t="str">
         <f>"&lt;Item&gt;
             &lt;ItemLink&gt;" &amp; B32 &amp; "&lt;/ItemLink&gt;
         &lt;/Item&gt;"</f>
         <v>&lt;Item&gt;
-            &lt;ItemLink&gt;1404000893&lt;/ItemLink&gt;
+            &lt;ItemLink&gt;1404000913&lt;/ItemLink&gt;
         &lt;/Item&gt;</v>
       </c>
       <c r="D32" t="s">
-        <v>56</v>
+        <v>98</v>
       </c>
       <c r="E32" t="s">
         <v>9</v>
@@ -1819,27 +1795,27 @@
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>75</v>
+        <v>102</v>
       </c>
       <c r="B33" t="s">
-        <v>76</v>
+        <v>103</v>
       </c>
       <c r="C33" t="str">
         <f>"&lt;Item&gt;
             &lt;ItemLink&gt;" &amp; B33 &amp; "&lt;/ItemLink&gt;
         &lt;/Item&gt;"</f>
         <v>&lt;Item&gt;
-            &lt;ItemLink&gt;1404000898&lt;/ItemLink&gt;
+            &lt;ItemLink&gt;1404000915&lt;/ItemLink&gt;
         &lt;/Item&gt;</v>
       </c>
       <c r="D33" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
       <c r="E33" t="s">
         <v>9</v>
       </c>
       <c r="F33" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G33" t="s">
         <v>9</v>
@@ -1850,27 +1826,27 @@
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>63</v>
+        <v>117</v>
       </c>
       <c r="B34" t="s">
-        <v>64</v>
+        <v>118</v>
       </c>
       <c r="C34" t="str">
         <f>"&lt;Item&gt;
             &lt;ItemLink&gt;" &amp; B34 &amp; "&lt;/ItemLink&gt;
         &lt;/Item&gt;"</f>
         <v>&lt;Item&gt;
-            &lt;ItemLink&gt;1404000901&lt;/ItemLink&gt;
+            &lt;ItemLink&gt;1404000916&lt;/ItemLink&gt;
         &lt;/Item&gt;</v>
       </c>
       <c r="D34" t="s">
-        <v>65</v>
+        <v>119</v>
       </c>
       <c r="E34" t="s">
         <v>9</v>
       </c>
       <c r="F34" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="G34" t="s">
         <v>9</v>
@@ -1881,27 +1857,27 @@
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>96</v>
+        <v>66</v>
       </c>
       <c r="B35" t="s">
-        <v>97</v>
+        <v>67</v>
       </c>
       <c r="C35" t="str">
         <f>"&lt;Item&gt;
             &lt;ItemLink&gt;" &amp; B35 &amp; "&lt;/ItemLink&gt;
         &lt;/Item&gt;"</f>
         <v>&lt;Item&gt;
-            &lt;ItemLink&gt;1404000913&lt;/ItemLink&gt;
+            &lt;ItemLink&gt;1404000917&lt;/ItemLink&gt;
         &lt;/Item&gt;</v>
       </c>
       <c r="D35" t="s">
-        <v>98</v>
+        <v>68</v>
       </c>
       <c r="E35" t="s">
         <v>9</v>
       </c>
       <c r="F35" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G35" t="s">
         <v>9</v>
@@ -1943,27 +1919,27 @@
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>14</v>
+        <v>51</v>
       </c>
       <c r="B37" t="s">
-        <v>15</v>
+        <v>52</v>
       </c>
       <c r="C37" t="str">
         <f>"&lt;Item&gt;
             &lt;ItemLink&gt;" &amp; B37 &amp; "&lt;/ItemLink&gt;
         &lt;/Item&gt;"</f>
         <v>&lt;Item&gt;
-            &lt;ItemLink&gt;1404000923&lt;/ItemLink&gt;
+            &lt;ItemLink&gt;1404000922&lt;/ItemLink&gt;
         &lt;/Item&gt;</v>
       </c>
       <c r="D37" t="s">
-        <v>16</v>
+        <v>53</v>
       </c>
       <c r="E37" t="s">
         <v>9</v>
       </c>
       <c r="F37" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="G37" t="s">
         <v>9</v>
@@ -1974,21 +1950,21 @@
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B38" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C38" t="str">
         <f>"&lt;Item&gt;
             &lt;ItemLink&gt;" &amp; B38 &amp; "&lt;/ItemLink&gt;
         &lt;/Item&gt;"</f>
         <v>&lt;Item&gt;
-            &lt;ItemLink&gt;1404000924&lt;/ItemLink&gt;
+            &lt;ItemLink&gt;1404000923&lt;/ItemLink&gt;
         &lt;/Item&gt;</v>
       </c>
       <c r="D38" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="E38" t="s">
         <v>9</v>
@@ -2005,27 +1981,27 @@
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="B39" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="C39" t="str">
         <f>"&lt;Item&gt;
             &lt;ItemLink&gt;" &amp; B39 &amp; "&lt;/ItemLink&gt;
         &lt;/Item&gt;"</f>
         <v>&lt;Item&gt;
-            &lt;ItemLink&gt;1404000926&lt;/ItemLink&gt;
+            &lt;ItemLink&gt;1404000924&lt;/ItemLink&gt;
         &lt;/Item&gt;</v>
       </c>
       <c r="D39" t="s">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="E39" t="s">
         <v>9</v>
       </c>
       <c r="F39" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G39" t="s">
         <v>9</v>
@@ -2036,27 +2012,27 @@
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="B40" t="s">
-        <v>52</v>
+        <v>21</v>
       </c>
       <c r="C40" t="str">
         <f>"&lt;Item&gt;
             &lt;ItemLink&gt;" &amp; B40 &amp; "&lt;/ItemLink&gt;
         &lt;/Item&gt;"</f>
         <v>&lt;Item&gt;
-            &lt;ItemLink&gt;1404000922&lt;/ItemLink&gt;
+            &lt;ItemLink&gt;1404000926&lt;/ItemLink&gt;
         &lt;/Item&gt;</v>
       </c>
       <c r="D40" t="s">
-        <v>53</v>
+        <v>22</v>
       </c>
       <c r="E40" t="s">
         <v>9</v>
       </c>
       <c r="F40" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="G40" t="s">
         <v>9</v>
@@ -2166,7 +2142,7 @@
       </filters>
     </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A15:H43">
-      <sortCondition ref="H1:H43"/>
+      <sortCondition ref="B1:B43"/>
     </sortState>
   </autoFilter>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>